<commit_message>
docs: cierra la cobertura del libro de modulos y pone subtarea de QA en cada historia
Las 88 funcionalidades de las hojas M-01 a M-13 quedan con historia asignada:
18 no la tenían, doce ya estaban cubiertas por un ítem del Sprint 5 sin trazar
y seis necesitaron historia nueva (CONS-46, VAL-19 a VAL-22, TEC-21).

Se corrigen 16 etiquetas de requisito que no aparecían en ninguna fila, de modo
que los 36 RF, los 11 RNF y las 5 REST del SRS quedan trazados a funcionalidad
e historia. Cada historia lleva su subtarea QA-<id>: QA revisa la evidencia y
cierra, según GOBIERNO_DEL_EQUIPO.md §2.3.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wiki/05-backlog/MANI_MODULOS_SERVICIOS_Y_BACKLOG_S5.xlsx
+++ b/wiki/05-backlog/MANI_MODULOS_SERVICIOS_Y_BACKLOG_S5.xlsx
@@ -38,6 +38,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Criterios transversales S4" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Criterios por historia S4" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Criterios US-02.1.1" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Cierre de cobertura" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Gestion del sprint" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Subtareas de QA" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,7 +94,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -131,6 +134,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -218,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -287,6 +300,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1366,7 +1391,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>RF-15 / RF-17</t>
+          <t>RF-34 / RF-15 / RF-17</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1419,7 +1444,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>RNF-03</t>
+          <t>RF-35 / RNF-03</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1676,7 +1701,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-30</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1776,7 +1801,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>RF-02 / RNF-10</t>
+          <t>RF-33 / RF-02 / RNF-10</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1828,7 +1853,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>RF-18</t>
+          <t>RF-36 / RF-18</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1880,7 +1905,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>RF-18</t>
+          <t>RF-36 / RF-18</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -2033,7 +2058,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-35 · TEC-01</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -2691,7 +2716,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>RF-24</t>
+          <t>RF-24 / REST-03</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2743,7 +2768,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>RF-24</t>
+          <t>RF-24 / RNF-06 / RNF-11 / REST-03</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -3004,7 +3029,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>RF-25</t>
+          <t>RF-25 / RNF-10 / REST-05</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -12003,7 +12028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12019,6 +12044,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -12033,6 +12059,7 @@
       <c r="C3" s="19" t="n"/>
       <c r="D3" s="20" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
@@ -12096,6 +12123,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -12137,10 +12165,10 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -12155,10 +12183,10 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
@@ -12173,98 +12201,117 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>Gestion (SM, PO)</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Facilitacion del sprint y validacion final del producto</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="26" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr"/>
-      <c r="C20" s="21" t="n">
-        <v>83</v>
-      </c>
-      <c r="D20" s="21" t="n">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="21" t="n">
+        <v>91</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Orden sugerido de ejecucion</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>1. Desbloquear el ambiente: TEC-09, TEC-10, TEC-11 y TEC-16. Sin token real ES256 ni QA sembrada, ningun video vale.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="21" customHeight="1">
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>2. Decisiones de Mesa que bloquean codigo: TEC-01, TEC-12, y las salidas de P-5 y P-6.</t>
+          <t>1. Desbloquear el ambiente: TEC-09, TEC-10, TEC-11 y TEC-16. Sin token real ES256 ni QA sembrada, ningun video vale.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="21" customHeight="1">
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>3. Arreglar los defectos de despacho antes de grabar: TEC-02, TEC-03, TEC-04, TEC-05, TEC-06.</t>
+          <t>2. Decisiones de Mesa que bloquean codigo: TEC-01, TEC-12, y las salidas de P-5 y P-6.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="21" customHeight="1">
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>4. Migrar el front al Gateway: CONS-03 y TEC-18, que habilitan VAL-10 a VAL-14.</t>
+          <t>3. Arreglar los defectos de despacho antes de grabar: TEC-02, TEC-03, TEC-04, TEC-05, TEC-06.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="21" customHeight="1">
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>5. Grabar la tanda de validacion VAL-01 a VAL-18, abriendo bug con minuto exacto por cada fallo.</t>
+          <t>4. Migrar el front al Gateway: CONS-03 y TEC-18, que habilitan VAL-10 a VAL-14.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1">
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>6. Construir el shell y la sesion: CONS-01, CONS-02, CONS-07 a CONS-09, luego VAL-17.</t>
+          <t>5. Grabar la tanda de validacion VAL-01 a VAL-18, abriendo bug con minuto exacto por cada fallo.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1">
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>7. Mocks que habilitan front: CONS-35 (notificaciones) y CONS-38 (pasarela).</t>
+          <t>6. Construir el shell y la sesion: CONS-01, CONS-02, CONS-07 a CONS-09, luego VAL-17.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="21" customHeight="1">
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>8. Rules Service: TEC-15 y CONS-18, que desbloquean tarifario, alertas y ranking.</t>
+          <t>7. Mocks que habilitan front: CONS-35 (notificaciones) y CONS-38 (pasarela).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="21" customHeight="1">
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>9. Resto del ciclo del servicio: cotizacion, ejecucion, calificacion y comunicacion.</t>
+          <t>8. Rules Service: TEC-15 y CONS-18, que desbloquean tarifario, alertas y ranking.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="21" customHeight="1">
       <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>9. Resto del ciclo del servicio: cotizacion, ejecucion, calificacion y comunicacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>10. Modularizacion CONS-10 y CONS-11 al final, cuando las pruebas ya cubren el comportamiento.</t>
         </is>
@@ -12303,7 +12350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13219,6 +13266,206 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>VAL-19</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>M-03</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Validar el contrato del perfil del aliado que consumen Dispatch y Rules</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Existe en codigo pero nunca se valido como contrato. Pedir el perfil del aliado por el Gateway con token real ES256 y comprobar: responde los campos que Dispatch y Rules declaran consumir, no expone documentos KYC ni datos de otro aliado, y con el token de un aliado del tenant B sobre un aliado del tenant A responde 403 o 404 y nunca 200 con datos. Video desde el front o, si no tiene pantalla, corrida Newman adjunta.</t>
+        </is>
+      </c>
+      <c r="F25" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="inlineStr">
+        <is>
+          <t>TEC-10 (token real ES256)</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>CORE, DISPATCH, RULES</t>
+        </is>
+      </c>
+      <c r="J25" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>VAL-20</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>M-04</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Validar que el catalogo responde solo las categorias y zonas del tenant del claim</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Cliente / Aliado</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Implementado y sin validar. Consultar el catalogo por el Gateway con usuarios de dos tenants y comprobar que cada uno ve solo sus categorias activas, que una categoria desactivada no aparece, y que el tenant no se puede forzar por cuerpo ni por cabecera (se toma del claim, T4). El catalogo es pre-auth en nginx: comprobar tambien que sin token no filtra datos de ningun tenant.</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" s="26" t="inlineStr">
+        <is>
+          <t>TEC-10, TEC-16</t>
+        </is>
+      </c>
+      <c r="I26" s="26" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="J26" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>VAL-21</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Validar el contexto de solicitud que Dispatch pide a Core</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>Implementado y sin validar. Comprobar que Dispatch obtiene zona, categoria y estado de la solicitud por HTTP a Core y no por SQL sobre tablas de Core (T1), que si Core no responde Dispatch devuelve 503 y no arma el contexto con logica local (T2), y que el contexto de una solicitud del tenant A nunca se entrega con el token del tenant B.</t>
+        </is>
+      </c>
+      <c r="F27" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H27" s="26" t="inlineStr">
+        <is>
+          <t>TEC-02, TEC-10</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="inlineStr">
+        <is>
+          <t>CORE, DISPATCH</t>
+        </is>
+      </c>
+      <c r="J27" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>VAL-22</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Validar idempotencia de la creacion de solicitud y del despacho bajo reintento</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>RNF-03 exige que las operaciones criticas resistan reintentos sin duplicar. Comprobar: reintento con la misma claveIdempotencia no crea una segunda solicitud; reintento de la orquestacion no duplica el broadcast; y tras un corte parcial del broadcast el reintento completa las ofertas que faltan en vez de congelarse, que es el defecto D-4. Requiere TEC-04 desplegado.</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" s="26" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="H28" s="26" t="inlineStr">
+        <is>
+          <t>TEC-04 (paginar y rehacer la guarda de idempotencia)</t>
+        </is>
+      </c>
+      <c r="I28" s="26" t="inlineStr">
+        <is>
+          <t>CORE, DISPATCH</t>
+        </is>
+      </c>
+      <c r="J28" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
@@ -13234,7 +13481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15392,6 +15639,56 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="28" t="inlineStr">
+        <is>
+          <t>CONS-46</t>
+        </is>
+      </c>
+      <c r="B52" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>Alta y administracion de tenants por el administrador de plataforma</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Admin de plataforma</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="inlineStr">
+        <is>
+          <t>RF-01 es critico y hoy solo existe GET /api/v1/core/tenants: no hay forma de crear un tenant por la aplicacion. End to end desde cero: pantalla de administracion de plataforma, alta del tenant con su slug y sus datos, edicion, y consulta del listado. El alta crea el tenant aislado: sus tablas nacen con tenant_id y su politica por tenant en la misma migracion (T3). Solo el administrador de plataforma puede crear tenants; un admin de tenant que lo intente recibe 403. Queda registrado quien lo creo, cuando y con que correlationId (T10). No incluye el estado del tenant, que es CONS-43.</t>
+        </is>
+      </c>
+      <c r="F52" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="G52" s="26" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="H52" s="26" t="inlineStr">
+        <is>
+          <t>CONS-07 (shell), TEC-10</t>
+        </is>
+      </c>
+      <c r="I52" s="26" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="J52" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
@@ -15407,7 +15704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16386,6 +16683,51 @@
       <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Total: 20 tareas · 85 story points</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>TEC-21</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>Retirar BYPASSRLS: Core y Dispatch conectan con un rol de servicio sin privilegio de salto</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Seguridad / Migracion</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>BUG-SEC-02, R-09, R-06</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="26" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="G27" s="26" t="inlineStr">
+        <is>
+          <t>Core y DevOps</t>
+        </is>
+      </c>
+      <c r="H27" s="26" t="inlineStr">
+        <is>
+          <t>TEC-13 (identidad de servicio)</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="inlineStr">
+        <is>
+          <t>Hoy Core usa service_role o postgres y Dispatch usa postgres, los tres con BYPASSRLS, asi que ninguna politica RLS se evalua y el aislamiento de RNF-01 descansa solo en el codigo. Cerrar: cada servicio conecta con un rol propio sin BYPASSRLS; las 15 politicas tenant_isolation_* dejan de estar TO public (R-06); y una prueba demuestra que, con el filtro de aplicacion desactivado a proposito, la politica sigue bloqueando el acceso cruzado. Sin esto, VAL-16 no demuestra aislamiento real sino aislamiento por codigo.</t>
         </is>
       </c>
     </row>
@@ -23530,6 +23872,3533 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="92" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>Cierre de cobertura: cada funcionalidad con su historia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="86" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Revision del 24-oct-2026. Las 88 funcionalidades de las hojas M-01 a M-13 tienen ahora una historia asignada: 18 no la tenian. Doce ya estaban cubiertas por un item del Sprint 5 pero sin trazar en la columna Historia; seis necesitaron historia nueva (VAL-19 a VAL-22, CONS-46 y TEC-21). Regla aplicada: lo que no existe se construye end to end desde cero; lo que figura como implementado se valida contra lo pedido, porque un estado Done sin video por el Gateway con token real no acredita nada (SAD §7.5). Ademas se corrigieron 16 etiquetas de requisito: RF-29 a RF-36, RNF-06, RNF-07, RNF-11, REST-03 y REST-05 no aparecian en ninguna fila aunque su funcionalidad si existia. Ahora los 36 RF, los 11 RNF y las 5 REST del SRS estan trazados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Funcionalidad</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Modulo</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>RF / RNF</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Estado hoy</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>HU que la cubre</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>Tipo de HU</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>Que exige esa HU</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>M-01.1</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Registrar y administrar empresas (tenants)</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>RF-01</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Parcial: solo existe GET /core/tenants</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>CONS-46</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>Nueva · construccion desde 0</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>RF-01 es critico y no hay forma de crear un tenant por la aplicacion. Pantalla de administracion de plataforma con alta, edicion y listado; el alta crea el tenant aislado con tenant_id y politica en la misma migracion (T3); solo el admin de plataforma puede crear y queda registrado quien, cuando y el correlationId (T10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>M-01.2</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Aislamiento estricto de datos y archivos por tenant</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>RNF-01 / REST-04</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Parcial con defecto abierto</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>VAL-16 · TEC-21</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>Existente + tarea nueva</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>VAL-16 ya valida el aislamiento, pero hoy Core y Dispatch conectan con BYPASSRLS y ninguna politica RLS se evalua: el aislamiento descansa solo en el codigo. TEC-21 retira BYPASSRLS y quita el TO public de las 15 politicas, para que VAL-16 demuestre aislamiento real y no aislamiento por codigo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>M-01.3</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Configurar reglas operativas propias por tenant</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>RF-02 / RNF-02 / RNF-10 / REST-05</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente: Rules no existe</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>CONS-44 · TEC-15</t>
+        </is>
+      </c>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>RF-02 es critico y RNF-02 exige configurar sin nuevo despliegue. TEC-15 crea el repositorio del Rules Service y CONS-44 construye la configuracion por tenant. Hasta entonces ninguna regla es configurable y RNF-02 no se cumple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>M-01.4</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Identificacion de tenant no falsificable</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>RNF-01 / ADR-0018</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Implementado con defecto abierto</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>VAL-16 · TEC-09</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>El perimetro resuelve el tenant por auth_request y Core lo revalida, pero dev-token firmaba tenant_id y rol arbitrarios. TEC-09 cierra dev-token y VAL-16 comprueba que el tenant no se puede forzar por cuerpo ni por cabecera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>M-01.5</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Propiedad del esquema y de las migraciones en un solo servicio</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>M-01</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>ADR-0030 §1</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>TEC-08</t>
+        </is>
+      </c>
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>Existente, sin trazar</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="inlineStr">
+        <is>
+          <t>La conformidad esta comprobada: MANI-.NET no versiona DDL. Lo unico abierto es D-10, que la numeracion de migraciones salta de 0010 a 0013 sin registro del motivo, y eso lo cierra TEC-08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>M-02.1</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Inicio de sesion</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>M-02</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>RF-03</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Done sin validar en arquitectura vigente</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>VAL-01 · TEC-10</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>Figura Done pero nunca se ejecuto por el Gateway con un token real: el perimetro aceptaba solo HS256 y MANI-QA emite ES256. TEC-10 ya dejo un solo validador con ES256 y VAL-01 graba el login real de extremo a extremo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>M-02.10</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Recuperacion segura de contrasena</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>M-02</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>RF-04</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>CONS-04</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="inlineStr">
+        <is>
+          <t>Existente, sin trazar</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="inlineStr">
+        <is>
+          <t>RF-04 es de prioridad alta y no hay nada construido. CONS-04 lo construye desde cero contra Supabase Auth orquestado por Core, con el enlace de un solo uso y sin exponer si el correo existe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>M-02.13</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Validacion perimetral del token y propagacion de claims</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>M-02</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>RF-03</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Implementado con defecto abierto</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>VAL-18 · TEC-10</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="inlineStr">
+        <is>
+          <t>Habia dos validadores con politicas distintas y el perimetro era mas estricto que el interior. TEC-10 unifica en un solo validador; VAL-18 ejecuta la regresion de seguridad: token ausente, mal formado, alterado, vencido, con kid desconocido y con alg none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>M-02.14</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Autorizacion por rol y tenant en cada peticion</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>M-02</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>RF-03</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>VAL-18 · TEC-07</t>
+        </is>
+      </c>
+      <c r="G13" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="inlineStr">
+        <is>
+          <t>Implementado en Core, pero JwtAuthHelper de Dispatch caia a claims planos mientras Core prohibe ese respaldo: dos politicas de token en el mismo sistema. TEC-07 las unifica y VAL-18 comprueba que un rol insuficiente recibe 403 en los tres servicios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>M-03.6</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Perfil del aliado autenticado consumible por otros servicios</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>M-03</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>RF-30 / RF-05</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Implementado, nunca validado como contrato</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>VAL-19</t>
+        </is>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>Nueva · validacion</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>Existe en codigo y no figuraba ni en el cuerpo del PR que lo introdujo. VAL-19 lo valida como contrato: responde los campos que Dispatch y Rules declaran consumir, no expone documentos KYC, y con el token de otro tenant responde 403 o 404, nunca 200 con datos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>M-04.4</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Catalogo jerarquico de zonas geograficas</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>M-04</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>REST-01 / RNF-09</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>CONS-12</t>
+        </is>
+      </c>
+      <c r="G15" s="26" t="inlineStr">
+        <is>
+          <t>Existente, sin trazar</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="inlineStr">
+        <is>
+          <t>REST-01 y RNF-09 exigen cobertura por zonas de un catalogo jerarquico y nunca por radio. Falta el nivel de barrio, que es el mas fino del MVP, y eso lo construye CONS-12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>M-04.5</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Consulta del catalogo por tenant</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>M-04</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>RF-10</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Implementado, sin validar</t>
+        </is>
+      </c>
+      <c r="F16" s="29" t="inlineStr">
+        <is>
+          <t>VAL-20</t>
+        </is>
+      </c>
+      <c r="G16" s="26" t="inlineStr">
+        <is>
+          <t>Nueva · validacion</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="inlineStr">
+        <is>
+          <t>El catalogo es pre-auth en nginx, asi que hay que comprobar dos cosas distintas: que con token cada tenant ve solo sus categorias activas y no puede forzar el tenant, y que sin token no filtra datos de ningun tenant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>M-05.3</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Contexto de la solicitud (zona, categoria, estado)</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>RF-12</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>Implementado, sin validar</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>VAL-21</t>
+        </is>
+      </c>
+      <c r="G17" s="26" t="inlineStr">
+        <is>
+          <t>Nueva · validacion</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="inlineStr">
+        <is>
+          <t>VAL-21 comprueba que Dispatch obtiene el contexto por HTTP a Core y no por SQL sobre tablas de Core (T1), que si Core no responde devuelve 503 sin logica local (T2), y que el contexto del tenant A nunca se entrega con el token del tenant B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>M-05.6</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Broadcast de ofertas a los aliados elegibles</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>RF-14</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>VAL-15 · TEC-04</t>
+        </is>
+      </c>
+      <c r="G18" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="inlineStr">
+        <is>
+          <t>El broadcast pide PageSize=50 sin recorrer paginas y descarta totalCount, asi que con mas de 50 elegibles no oferta a todos. TEC-04 lo pagina y rehace la guarda de idempotencia; VAL-15 graba el broadcast completo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>M-05.8</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>Rechazar oferta</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>RF-14</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>VAL-14 · TEC-03</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="inlineStr">
+        <is>
+          <t>La politica solicitud_rechazo_aliado lee la tabla aliado y Dispatch no tiene SELECT sobre ella, asi que el INSERT falla con permission denied. TEC-03 corrige la politica y VAL-14 graba el rechazo y comprueba que la solicitud sigue disponible para los demas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>M-05.9</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Idempotencia de la creacion y del despacho</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>M-05</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>RNF-03</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F20" s="29" t="inlineStr">
+        <is>
+          <t>VAL-22 · TEC-04</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="inlineStr">
+        <is>
+          <t>Nueva validacion + tarea existente</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="inlineStr">
+        <is>
+          <t>RNF-03 exige que las operaciones criticas resistan reintentos sin duplicar. Hoy la guarda existingOffers.Count&gt;0 congela el reintento tras un corte parcial. TEC-04 la rehace y VAL-22 comprueba los tres casos: misma claveIdempotencia, reintento de la orquestacion y corte parcial del broadcast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>M-08.3</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>Cierre condicionado a la calificacion bidireccional</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>M-08</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>RF-19</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>CONS-30</t>
+        </is>
+      </c>
+      <c r="G21" s="26" t="inlineStr">
+        <is>
+          <t>Existente, sin trazar</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="inlineStr">
+        <is>
+          <t>RF-19 exige que el servicio no pueda cerrarse hasta que ambas partes califiquen. CONS-30 lo construye desde cero, con la calificacion de las dos partes como condicion de cierre y no como paso opcional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>M-09.1</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Frontera de notificacion del backend</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>M-09</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>RF-20</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="inlineStr">
+        <is>
+          <t>CONS-35 · TEC-01</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="inlineStr">
+        <is>
+          <t>Existentes, sin trazar</t>
+        </is>
+      </c>
+      <c r="H22" s="26" t="inlineStr">
+        <is>
+          <t>Dispatch no debe insertar en tablas de notificacion: notifica a traves de Core (T1). El pendiente P-4 del SAD §7.4 sobre quien es dueno de la frontera sigue abierto y lo cierra TEC-01; CONS-35 construye el mock del proveedor push para que el front exista.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="96" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>Sprint 5 · Historias de gestion: Scrum Master y Product Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="76" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Dos historias que no son de desarrollo y que el sprint necesita igual. SM-01 es la facilitacion del sprint, que hoy no esta en ningun bloque aunque la Scrum Master la ejecuta. PO-01 es la validacion del producto al final: es la que cierra el sprint, porque el DoD exige que cada funcionalidad este demostrada por video y aceptada, y alguien tiene que dar esa aceptacion. Autoridad: el PO decide los criterios de aceptacion y QA decide el DoD (GOBIERNO_DEL_EQUIPO.md §2.3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Criterios de aceptacion</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>Dependencias</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>Momento</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>SM-01</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Facilitar el sprint y sostener la trazabilidad del tablero</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Sara Albarracin (Scrum Master)</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Ceremonias de la sesion 5 celebradas y registradas: planning con el compromiso del sprint, dailies, review con la demostracion por video y retro con acuerdos. Cada item VAL, CONS y TEC existe en Jira con su clave, su estimacion y su responsable. Los impedimentos quedan registrados con fecha de apertura, responsable y fecha de cierre. Los indicadores del sprint se publican al cierre. Ningun item se declara terminado sin la subtarea de QA cerrada.</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>Todo el sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>PO-01</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Validar el producto terminado y aceptar el incremento</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Camila Beltran (Product Owner)</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Recorrido completo del producto por el front, en QA y a traves del Gateway, con token real ES256, sobre el build desplegado. Se recorre el ciclo entero: registro, inicio de sesion por tipo, solicitud, elegibilidad, aceptacion sin doble asignacion, cotizacion, ejecucion, calificacion y cierre. Por cada funcionalidad del libro de modulos el PO declara aceptada o rechazada contra su criterio de §6 del backlog, no contra el estado del tablero. Un rechazo abre bug con el minuto exacto del video. El acta de aceptacion lista que se acepta, que se rechaza y que queda fuera del incremento con su causa (GOBIERNO_DEL_EQUIPO.md §10, incremento no entregado). Sin esta aceptacion el sprint no se cierra.</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>Todas las VAL y las CONS del sprint</t>
+        </is>
+      </c>
+      <c r="H6" s="26" t="inlineStr">
+        <is>
+          <t>Ultimos dias del sprint</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="104" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>Una subtarea de QA por historia: revisar y cerrar en Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Acuerdo del 24-oct-2026: ninguna historia pasa a Done por si misma. Cada una lleva una subtarea de Santiago (QA) que revisa la evidencia contra los criterios de la historia y es quien la mueve a Done. QA decide el DoD (GOBIERNO_DEL_EQUIPO.md §2.3), asi que la subtarea es el punto de control: si la evidencia no cumple, la historia vuelve y no se cierra. Esto cierra el hueco del Sprint 4, donde 14 subtareas de QA existian pero tres historias (SCRUM-1063, 1066 y 1068) no tenian ninguna, pendiente PE4 de §6.5 del backlog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Subtarea</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Bloque</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Titulo de la historia</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Que revisa y cierra QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-01</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>VAL-01</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Validar inicio de sesion con token real ES256 de extremo a extremo</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-02</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>VAL-02</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Validar registro de aliado persona natural por el camino Gateway-Core</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-03</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>VAL-03</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Validar registro de aliado empresa</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-04</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>VAL-04</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Validar registro de cliente persona natural</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-05</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>VAL-05</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Validar edicion del perfil propio</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-06</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>VAL-06</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Validar aprobacion y rechazo de aliado en la bandeja de verificacion</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-07</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>VAL-07</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Validar declaracion de cobertura por zonas del aliado</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-08</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>VAL-08</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Validar que el aliado declara las categorias que atiende</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-09</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>VAL-09</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Validar gestion de categorias del tenant</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-10</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>VAL-10</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Validar creacion de la solicitud en Core desde el front</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-11</t>
+        </is>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>VAL-11</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Validar elegibilidad de aliados por categoria, zona, disponibilidad y rechazo previo</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-12</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>VAL-12</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Validar filtro por tipo de aliado</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-13</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>VAL-13</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>Validar aceptacion sin doble asignacion con dos aliados simultaneos</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-14</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>VAL-14</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Validar rechazo de oferta</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-15</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>VAL-15</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>Validar broadcast de ofertas y notificacion por la frontera de Core</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-16</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>VAL-16</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Validar aislamiento multi-tenant endpoint por endpoint</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-17</t>
+        </is>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
+        <is>
+          <t>VAL-17</t>
+        </is>
+      </c>
+      <c r="C21" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>Validar logout y expiracion de sesion</t>
+        </is>
+      </c>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-18</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>VAL-18</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Ejecutar la regresion de seguridad de identidad (17 casos negativos y 1 positivo)</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-19</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
+        <is>
+          <t>VAL-19</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>Validar el contrato del perfil del aliado que consumen Dispatch y Rules</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-20</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>VAL-20</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Validar que el catalogo responde solo las categorias y zonas del tenant del claim</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-21</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>VAL-21</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>Validar el contexto de solicitud que Dispatch pide a Core</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>QA-VAL-22</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>VAL-22</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Validacion</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Validar idempotencia de la creacion de solicitud y del despacho bajo reintento</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el video existe, que se grabo desde el front y no desde Postman ni consola, que corre en QA por el Gateway, que el token es real ES256 y no dev-token, que se ve el usuario y el rol con el que entra, la accion completa y el resultado persistido al recargar, y que incluye el caso negativo de aislamiento. Duracion maxima 4 minutos sin cortes en el tramo de persistencia. Evidencia enlazada con el SHA desplegado y la fecha. Si falta cualquiera de estos, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-01</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
+        <is>
+          <t>CONS-01</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>Inicio de sesion separado por tipo de usuario</t>
+        </is>
+      </c>
+      <c r="E27" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-02</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>CONS-02</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Logout</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-03</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>CONS-03</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>Autenticacion consumida desde la API y retiro de Supabase directo en el cliente</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-04</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>CONS-04</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Recuperacion segura de contrasena</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-05</t>
+        </is>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
+        <is>
+          <t>CONS-05</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D31" s="26" t="inlineStr">
+        <is>
+          <t>Registro de cliente empresa</t>
+        </is>
+      </c>
+      <c r="E31" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-06</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>CONS-06</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Registro de empleado directo</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-07</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>CONS-07</t>
+        </is>
+      </c>
+      <c r="C33" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>Menu superior por rol con sesion visible</t>
+        </is>
+      </c>
+      <c r="E33" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-08</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>CONS-08</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Pantalla de inicio por tipo de usuario</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-09</t>
+        </is>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
+        <is>
+          <t>CONS-09</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>Enrutamiento por rol con guardas de sesion</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-10</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>CONS-10</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Dividir el front en modulos independientes por dominio</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-11</t>
+        </is>
+      </c>
+      <c r="B37" s="26" t="inlineStr">
+        <is>
+          <t>CONS-11</t>
+        </is>
+      </c>
+      <c r="C37" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>Dividir el Core por dominios internos</t>
+        </is>
+      </c>
+      <c r="E37" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-12</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>CONS-12</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Barrios como nivel mas fino del catalogo de zonas</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-13</t>
+        </is>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
+        <is>
+          <t>CONS-13</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>Visualizacion en mapa de zonas, barrios y sitio de servicio</t>
+        </is>
+      </c>
+      <c r="E39" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-14</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>CONS-14</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Activar y desactivar categoria sin afectar servicios en curso</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-15</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>CONS-15</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Aliado gestiona su disponibilidad y sus ausencias</t>
+        </is>
+      </c>
+      <c r="E41" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-16</t>
+        </is>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>CONS-16</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>Cliente empresa administra multiples sitios de servicio</t>
+        </is>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-17</t>
+        </is>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>CONS-17</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Reglas contextuales del sitio visibles al aliado antes de programar</t>
+        </is>
+      </c>
+      <c r="E43" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-18</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>CONS-18</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Orden del listado de aliados en el Rules Service</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-19</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>CONS-19</t>
+        </is>
+      </c>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Priorizar solicitud por comision ofrecida</t>
+        </is>
+      </c>
+      <c r="E45" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-20</t>
+        </is>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>CONS-20</t>
+        </is>
+      </c>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Cancelar solicitud antes de la ejecucion</t>
+        </is>
+      </c>
+      <c r="E46" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-21</t>
+        </is>
+      </c>
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>CONS-21</t>
+        </is>
+      </c>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>Cotizacion con mano de obra y materiales separados</t>
+        </is>
+      </c>
+      <c r="E47" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-22</t>
+        </is>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>CONS-22</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>Alerta de cotizacion fuera del rango del tarifario</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-23</t>
+        </is>
+      </c>
+      <c r="B49" s="26" t="inlineStr">
+        <is>
+          <t>CONS-23</t>
+        </is>
+      </c>
+      <c r="C49" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D49" s="26" t="inlineStr">
+        <is>
+          <t>Cliente acepta, rechaza o solicita ajuste de la cotizacion</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-24</t>
+        </is>
+      </c>
+      <c r="B50" s="26" t="inlineStr">
+        <is>
+          <t>CONS-24</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D50" s="26" t="inlineStr">
+        <is>
+          <t>Marcar inicio y fin de la ejecucion</t>
+        </is>
+      </c>
+      <c r="E50" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-25</t>
+        </is>
+      </c>
+      <c r="B51" s="26" t="inlineStr">
+        <is>
+          <t>CONS-25</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>Registrar eventos y observaciones durante la ejecucion</t>
+        </is>
+      </c>
+      <c r="E51" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-26</t>
+        </is>
+      </c>
+      <c r="B52" s="26" t="inlineStr">
+        <is>
+          <t>CONS-26</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>Registrar evidencias sin conexion y sincronizarlas</t>
+        </is>
+      </c>
+      <c r="E52" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-27</t>
+        </is>
+      </c>
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>CONS-27</t>
+        </is>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D53" s="26" t="inlineStr">
+        <is>
+          <t>Cargar la tabla de tarifas por categoria</t>
+        </is>
+      </c>
+      <c r="E53" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-28</t>
+        </is>
+      </c>
+      <c r="B54" s="26" t="inlineStr">
+        <is>
+          <t>CONS-28</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D54" s="26" t="inlineStr">
+        <is>
+          <t>Ver la tarifa de referencia al cotizar</t>
+        </is>
+      </c>
+      <c r="E54" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-29</t>
+        </is>
+      </c>
+      <c r="B55" s="26" t="inlineStr">
+        <is>
+          <t>CONS-29</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D55" s="26" t="inlineStr">
+        <is>
+          <t>Reporte de cotizaciones fuera de rango por periodo</t>
+        </is>
+      </c>
+      <c r="E55" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-30</t>
+        </is>
+      </c>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>CONS-30</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D56" s="26" t="inlineStr">
+        <is>
+          <t>Calificacion bidireccional y cierre condicionado</t>
+        </is>
+      </c>
+      <c r="E56" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-31</t>
+        </is>
+      </c>
+      <c r="B57" s="26" t="inlineStr">
+        <is>
+          <t>CONS-31</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>Calificacion agregada visible en el listado de aliados</t>
+        </is>
+      </c>
+      <c r="E57" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-32</t>
+        </is>
+      </c>
+      <c r="B58" s="26" t="inlineStr">
+        <is>
+          <t>CONS-32</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D58" s="26" t="inlineStr">
+        <is>
+          <t>Penalizacion por cancelacion tardia</t>
+        </is>
+      </c>
+      <c r="E58" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-33</t>
+        </is>
+      </c>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>CONS-33</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>Historial de servicios del cliente y de trabajos del aliado</t>
+        </is>
+      </c>
+      <c r="E59" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-34</t>
+        </is>
+      </c>
+      <c r="B60" s="26" t="inlineStr">
+        <is>
+          <t>CONS-34</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>Mensajeria cliente-aliado por servicio</t>
+        </is>
+      </c>
+      <c r="E60" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-35</t>
+        </is>
+      </c>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>CONS-35</t>
+        </is>
+      </c>
+      <c r="C61" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>Mock del proveedor de notificaciones push en el backend</t>
+        </is>
+      </c>
+      <c r="E61" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-36</t>
+        </is>
+      </c>
+      <c r="B62" s="26" t="inlineStr">
+        <is>
+          <t>CONS-36</t>
+        </is>
+      </c>
+      <c r="C62" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>Notificaciones de mensajes nuevos y del ciclo del servicio</t>
+        </is>
+      </c>
+      <c r="E62" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-37</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="inlineStr">
+        <is>
+          <t>CONS-37</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>Consultar la conversacion para atender una queja</t>
+        </is>
+      </c>
+      <c r="E63" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-38</t>
+        </is>
+      </c>
+      <c r="B64" s="26" t="inlineStr">
+        <is>
+          <t>CONS-38</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>Mock de la pasarela de pagos</t>
+        </is>
+      </c>
+      <c r="E64" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-39</t>
+        </is>
+      </c>
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>CONS-39</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>Registro inmutable de transacciones</t>
+        </is>
+      </c>
+      <c r="E65" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-40</t>
+        </is>
+      </c>
+      <c r="B66" s="26" t="inlineStr">
+        <is>
+          <t>CONS-40</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D66" s="26" t="inlineStr">
+        <is>
+          <t>Liquidacion al aliado con comision configurable</t>
+        </is>
+      </c>
+      <c r="E66" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-41</t>
+        </is>
+      </c>
+      <c r="B67" s="26" t="inlineStr">
+        <is>
+          <t>CONS-41</t>
+        </is>
+      </c>
+      <c r="C67" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>Registro y gestion de quejas</t>
+        </is>
+      </c>
+      <c r="E67" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-42</t>
+        </is>
+      </c>
+      <c r="B68" s="26" t="inlineStr">
+        <is>
+          <t>CONS-42</t>
+        </is>
+      </c>
+      <c r="C68" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D68" s="26" t="inlineStr">
+        <is>
+          <t>Metricas operativas por tenant y endpoint /metrics</t>
+        </is>
+      </c>
+      <c r="E68" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-43</t>
+        </is>
+      </c>
+      <c r="B69" s="26" t="inlineStr">
+        <is>
+          <t>CONS-43</t>
+        </is>
+      </c>
+      <c r="C69" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D69" s="26" t="inlineStr">
+        <is>
+          <t>Administrar el estado de los tenants</t>
+        </is>
+      </c>
+      <c r="E69" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-44</t>
+        </is>
+      </c>
+      <c r="B70" s="26" t="inlineStr">
+        <is>
+          <t>CONS-44</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D70" s="26" t="inlineStr">
+        <is>
+          <t>Configuracion de reglas por tenant sin despliegue</t>
+        </is>
+      </c>
+      <c r="E70" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-45</t>
+        </is>
+      </c>
+      <c r="B71" s="26" t="inlineStr">
+        <is>
+          <t>CONS-45</t>
+        </is>
+      </c>
+      <c r="C71" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D71" s="26" t="inlineStr">
+        <is>
+          <t>Cifrado y manejo de secretos verificado de punta a punta</t>
+        </is>
+      </c>
+      <c r="E71" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="31" t="inlineStr">
+        <is>
+          <t>QA-CONS-46</t>
+        </is>
+      </c>
+      <c r="B72" s="26" t="inlineStr">
+        <is>
+          <t>CONS-46</t>
+        </is>
+      </c>
+      <c r="C72" s="26" t="inlineStr">
+        <is>
+          <t>Construccion</t>
+        </is>
+      </c>
+      <c r="D72" s="26" t="inlineStr">
+        <is>
+          <t>Alta y administracion de tenants por el administrador de plataforma</t>
+        </is>
+      </c>
+      <c r="E72" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba los criterios de aceptacion de la historia uno por uno, los criterios transversales T1 a T10 que le apliquen, las pruebas automatizadas nuevas en verde, el Quality Gate de SonarQube del repositorio tocado y la evidencia de la ejecucion en QA por el Gateway con token real. Verifica tambien que lo construido cumple el requisito del SRS que la historia dice cubrir, no solo que el codigo exista. Si algo falta, la historia no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-01</t>
+        </is>
+      </c>
+      <c r="B73" s="26" t="inlineStr">
+        <is>
+          <t>TEC-01</t>
+        </is>
+      </c>
+      <c r="C73" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D73" s="26" t="inlineStr">
+        <is>
+          <t>Cerrar la contradiccion documental sobre quien crea la solicitud</t>
+        </is>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-02</t>
+        </is>
+      </c>
+      <c r="B74" s="26" t="inlineStr">
+        <is>
+          <t>TEC-02</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D74" s="26" t="inlineStr">
+        <is>
+          <t>Fijar el contexto de identidad en cada transaccion de Dispatch</t>
+        </is>
+      </c>
+      <c r="E74" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-03</t>
+        </is>
+      </c>
+      <c r="B75" s="26" t="inlineStr">
+        <is>
+          <t>TEC-03</t>
+        </is>
+      </c>
+      <c r="C75" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D75" s="26" t="inlineStr">
+        <is>
+          <t>Corregir la politica de solicitud_rechazo</t>
+        </is>
+      </c>
+      <c r="E75" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-04</t>
+        </is>
+      </c>
+      <c r="B76" s="26" t="inlineStr">
+        <is>
+          <t>TEC-04</t>
+        </is>
+      </c>
+      <c r="C76" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D76" s="26" t="inlineStr">
+        <is>
+          <t>Paginar el broadcast y hacer idempotente el reintento parcial</t>
+        </is>
+      </c>
+      <c r="E76" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-05</t>
+        </is>
+      </c>
+      <c r="B77" s="26" t="inlineStr">
+        <is>
+          <t>TEC-05</t>
+        </is>
+      </c>
+      <c r="C77" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D77" s="26" t="inlineStr">
+        <is>
+          <t>Distinguir conflicto de asignacion de conflicto de estado</t>
+        </is>
+      </c>
+      <c r="E77" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-06</t>
+        </is>
+      </c>
+      <c r="B78" s="26" t="inlineStr">
+        <is>
+          <t>TEC-06</t>
+        </is>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D78" s="26" t="inlineStr">
+        <is>
+          <t>Declarar CORE_SERVICE_URL en manifiestos versionados</t>
+        </is>
+      </c>
+      <c r="E78" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-07</t>
+        </is>
+      </c>
+      <c r="B79" s="26" t="inlineStr">
+        <is>
+          <t>TEC-07</t>
+        </is>
+      </c>
+      <c r="C79" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D79" s="26" t="inlineStr">
+        <is>
+          <t>Unificar la politica de token de Dispatch con la de Core</t>
+        </is>
+      </c>
+      <c r="E79" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-08</t>
+        </is>
+      </c>
+      <c r="B80" s="26" t="inlineStr">
+        <is>
+          <t>TEC-08</t>
+        </is>
+      </c>
+      <c r="C80" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D80" s="26" t="inlineStr">
+        <is>
+          <t>Documentar el salto de numeracion de migraciones y recuperar 0012</t>
+        </is>
+      </c>
+      <c r="E80" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-09</t>
+        </is>
+      </c>
+      <c r="B81" s="26" t="inlineStr">
+        <is>
+          <t>TEC-09</t>
+        </is>
+      </c>
+      <c r="C81" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D81" s="26" t="inlineStr">
+        <is>
+          <t>Cerrar dev-token y la ruta publica de validate-token en el Gateway, y rotar secretos</t>
+        </is>
+      </c>
+      <c r="E81" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-10</t>
+        </is>
+      </c>
+      <c r="B82" s="26" t="inlineStr">
+        <is>
+          <t>TEC-10</t>
+        </is>
+      </c>
+      <c r="C82" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D82" s="26" t="inlineStr">
+        <is>
+          <t>Un solo validador de token, con ES256, iss y aud</t>
+        </is>
+      </c>
+      <c r="E82" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-11</t>
+        </is>
+      </c>
+      <c r="B83" s="26" t="inlineStr">
+        <is>
+          <t>TEC-11</t>
+        </is>
+      </c>
+      <c r="C83" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D83" s="26" t="inlineStr">
+        <is>
+          <t>Confirmar o montar TLS en el borde</t>
+        </is>
+      </c>
+      <c r="E83" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-12</t>
+        </is>
+      </c>
+      <c r="B84" s="26" t="inlineStr">
+        <is>
+          <t>TEC-12</t>
+        </is>
+      </c>
+      <c r="C84" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D84" s="26" t="inlineStr">
+        <is>
+          <t>Ratificar ADR-0030 y ADR-0016 en Mesa</t>
+        </is>
+      </c>
+      <c r="E84" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-13</t>
+        </is>
+      </c>
+      <c r="B85" s="26" t="inlineStr">
+        <is>
+          <t>TEC-13</t>
+        </is>
+      </c>
+      <c r="C85" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D85" s="26" t="inlineStr">
+        <is>
+          <t>Definir identidad de servicio entre Dispatch y Core</t>
+        </is>
+      </c>
+      <c r="E85" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-14</t>
+        </is>
+      </c>
+      <c r="B86" s="26" t="inlineStr">
+        <is>
+          <t>TEC-14</t>
+        </is>
+      </c>
+      <c r="C86" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D86" s="26" t="inlineStr">
+        <is>
+          <t>Observabilidad minima de autenticacion</t>
+        </is>
+      </c>
+      <c r="E86" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-15</t>
+        </is>
+      </c>
+      <c r="B87" s="26" t="inlineStr">
+        <is>
+          <t>TEC-15</t>
+        </is>
+      </c>
+      <c r="C87" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D87" s="26" t="inlineStr">
+        <is>
+          <t>Crear el repositorio del Rules Service</t>
+        </is>
+      </c>
+      <c r="E87" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-16</t>
+        </is>
+      </c>
+      <c r="B88" s="26" t="inlineStr">
+        <is>
+          <t>TEC-16</t>
+        </is>
+      </c>
+      <c r="C88" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D88" s="26" t="inlineStr">
+        <is>
+          <t>Preparar el ambiente QA y los datos sembrados del sprint de validacion</t>
+        </is>
+      </c>
+      <c r="E88" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-17</t>
+        </is>
+      </c>
+      <c r="B89" s="26" t="inlineStr">
+        <is>
+          <t>TEC-17</t>
+        </is>
+      </c>
+      <c r="C89" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D89" s="26" t="inlineStr">
+        <is>
+          <t>Guia de grabacion y repositorio de videos</t>
+        </is>
+      </c>
+      <c r="E89" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-18</t>
+        </is>
+      </c>
+      <c r="B90" s="26" t="inlineStr">
+        <is>
+          <t>TEC-18</t>
+        </is>
+      </c>
+      <c r="C90" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D90" s="26" t="inlineStr">
+        <is>
+          <t>Migrar el front de solicitudes y asignacion al camino Gateway-Core</t>
+        </is>
+      </c>
+      <c r="E90" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-19</t>
+        </is>
+      </c>
+      <c r="B91" s="26" t="inlineStr">
+        <is>
+          <t>TEC-19</t>
+        </is>
+      </c>
+      <c r="C91" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D91" s="26" t="inlineStr">
+        <is>
+          <t>Migracion de usuario para direccion y foto de perfil</t>
+        </is>
+      </c>
+      <c r="E91" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-20</t>
+        </is>
+      </c>
+      <c r="B92" s="26" t="inlineStr">
+        <is>
+          <t>TEC-20</t>
+        </is>
+      </c>
+      <c r="C92" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D92" s="26" t="inlineStr">
+        <is>
+          <t>Persistir verificado_por en el adaptador real</t>
+        </is>
+      </c>
+      <c r="E92" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>QA-TEC-21</t>
+        </is>
+      </c>
+      <c r="B93" s="26" t="inlineStr">
+        <is>
+          <t>TEC-21</t>
+        </is>
+      </c>
+      <c r="C93" s="26" t="inlineStr">
+        <is>
+          <t>Tarea tecnica</t>
+        </is>
+      </c>
+      <c r="D93" s="26" t="inlineStr">
+        <is>
+          <t>Retirar BYPASSRLS: Core y Dispatch conectan con un rol de servicio sin privilegio de salto</t>
+        </is>
+      </c>
+      <c r="E93" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el hallazgo que la tarea dice cerrar ya no se reproduce en QA, con la corrida adjunta como evidencia, y que la correccion no rompio la regresion existente. Para las tareas de seguridad, comprueba ademas el caso negativo: que el vector cerrado efectivamente falla. Si el hallazgo sigue reproduciendose, la tarea no pasa a Done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="30" t="inlineStr">
+        <is>
+          <t>QA-SM-01</t>
+        </is>
+      </c>
+      <c r="B94" s="26" t="inlineStr">
+        <is>
+          <t>SM-01</t>
+        </is>
+      </c>
+      <c r="C94" s="26" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="D94" s="26" t="inlineStr">
+        <is>
+          <t>Sara Albarracin (Scrum Master)</t>
+        </is>
+      </c>
+      <c r="E94" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el registro existe y es verificable: para SM-01, que las ceremonias, los impedimentos y los indicadores estan publicados y que ningun item se declaro terminado sin su subtarea de QA cerrada; para PO-01, que el acta de aceptacion lista explicitamente lo aceptado, lo rechazado y lo que queda fuera del incremento con su causa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="30" t="inlineStr">
+        <is>
+          <t>QA-PO-01</t>
+        </is>
+      </c>
+      <c r="B95" s="26" t="inlineStr">
+        <is>
+          <t>PO-01</t>
+        </is>
+      </c>
+      <c r="C95" s="26" t="inlineStr">
+        <is>
+          <t>Gestion</t>
+        </is>
+      </c>
+      <c r="D95" s="26" t="inlineStr">
+        <is>
+          <t>Camila Beltran (Product Owner)</t>
+        </is>
+      </c>
+      <c r="E95" s="26" t="inlineStr">
+        <is>
+          <t>Comprueba que el registro existe y es verificable: para SM-01, que las ceremonias, los impedimentos y los indicadores estan publicados y que ningun item se declaro terminado sin su subtarea de QA cerrada; para PO-01, que el acta de aceptacion lista explicitamente lo aceptado, lo rechazado y lo que queda fuera del incremento con su causa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -24123,7 +27992,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-46</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -24175,7 +28044,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-16 · TEC-21</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -24224,12 +28093,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>RF-02 / RNF-02 / RNF-10</t>
+          <t>RF-02 / RNF-02 / RNF-10 / REST-05</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-44 · TEC-15</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -24282,7 +28151,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-16 · TEC-09</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -24334,7 +28203,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TEC-08</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -24482,7 +28351,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-01 · TEC-10</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -24893,7 +28762,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>RF-05 / RF-08</t>
+          <t>RF-30 / RF-05 / RF-08</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -24950,7 +28819,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-04</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -24997,7 +28866,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RF-31</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -25106,7 +28975,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-18 · TEC-10</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -25158,7 +29027,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-18 · TEC-07</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -25458,7 +29327,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>RF-12 (soporte)</t>
+          <t>RF-29 / RF-12 (soporte)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -25614,12 +29483,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>RF-05</t>
+          <t>RF-30 / RF-05</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-19</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -25925,7 +29794,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>CONS-12</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -25977,7 +29846,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-20</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -26278,7 +30147,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>RF-12</t>
+          <t>RF-12 / RNF-07</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -26336,7 +30205,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-21</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -26495,7 +30364,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-15 · TEC-04</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -26543,7 +30412,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>RF-14 / RNF-05</t>
+          <t>RF-14 / RNF-05 / RNF-07</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -26600,7 +30469,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-14 · TEC-03</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -26652,7 +30521,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VAL-22 · TEC-04</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -26700,7 +30569,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>RF-14</t>
+          <t>RF-32 / RF-14</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">

</xml_diff>

<commit_message>
[SCRUM-1469] Alinea el backlog V5 y el libro con el Sprint 5 de Jira
BACKLOG_MANI.md §0.3 y §0.4 se escribieron el 20-oct, antes del Planning.
Se ajustan a lo comprometido en Jira al 26-oct: responsables de las P0,
la P1 que no entró (SCRUM-864), la tabla de historias que entraron por
el Planning (antes «No entran») y la dependencia de SCRUM-866, que no
espera a SCRUM-1240 ni a crear el repositorio de Rules.

En el libro se corrigen tres celdas con criterio ya decidido: CONS-16 y
CONS-17 según la aprobación de la PO del 26-oct (SCRUM-1387 y 1388), y
la nota de M-06.2, que citaba mal el hallazgo D-5.

Quedan reportadas, sin resolver aquí, las contradicciones que decide el
PO o la SM: alcance de SCRUM-871 frente a SRS §1.2, SP distintos entre
Jira y el libro, y el momento de la modularización de Core.
</commit_message>
<xml_diff>
--- a/wiki/05-backlog/MANI_MODULOS_SERVICIOS_Y_BACKLOG_S5.xlsx
+++ b/wiki/05-backlog/MANI_MODULOS_SERVICIOS_Y_BACKLOG_S5.xlsx
@@ -1018,7 +1018,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Rules no existe (D-5)</t>
+          <t>Rules existe: MANI-Java esta en main desde el 21-oct con reglas de categoria reales (SCRUM-1070); /evaluate-rate y /rank-allies responden datos simulados. Falta el tarifario (CONS-27) y la validacion real contra el (CONS-22). D-5 es otro hueco: Dispatch no consulta a Rules para ordenar el listado.</t>
         </is>
       </c>
     </row>
@@ -12044,7 +12044,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -12059,7 +12058,6 @@
       <c r="C3" s="19" t="n"/>
       <c r="D3" s="20" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
@@ -12123,7 +12121,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -12239,7 +12236,6 @@
         <v>481</v>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
@@ -14275,7 +14271,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Alta, edicion y baja de sitios, cada uno con zona obligatoria.</t>
+          <t>Alta y edicion de sitios, cada uno con zona obligatoria. La baja queda pendiente de que la PO defina su semantica (estado o borrado logico), segun SCRUM-1387 (26-oct).</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
@@ -14321,7 +14317,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Reglas y condiciones del sitio mostradas en la oferta, antes de aceptar.</t>
+          <t>Reglas y condiciones del sitio visibles para el aliado asignado a una solicitud en ese sitio, antes de programar el servicio (criterio aprobado por la PO en SCRUM-1388 el 26-oct, tomado de SCRUM-853). Un aliado no asignado no las recibe.</t>
         </is>
       </c>
       <c r="F21" s="3" t="n">

</xml_diff>